<commit_message>
Copied fnuetz branch from gitlab
</commit_message>
<xml_diff>
--- a/src/pandaict/toolbox/template.xlsx
+++ b/src/pandaict/toolbox/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jringelstein\git\recode\pandaict\src\pandaict\toolbox\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75DCD2B8-35B7-46B8-A3EF-4592659B25EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ED42A3D-5F8B-41EB-AF74-989D88579235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3135" yWindow="2895" windowWidth="17280" windowHeight="9960" firstSheet="1" activeTab="2" xr2:uid="{6E993998-6D09-4908-A219-CC29AB846AA1}"/>
+    <workbookView xWindow="3960" yWindow="2565" windowWidth="18900" windowHeight="10965" activeTab="2" xr2:uid="{6E993998-6D09-4908-A219-CC29AB846AA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Howto" sheetId="17" r:id="rId1"/>
@@ -20,9 +20,9 @@
     <sheet name="Links" sheetId="11" r:id="rId5"/>
     <sheet name="Connections" sheetId="12" r:id="rId6"/>
     <sheet name="Apps" sheetId="13" r:id="rId7"/>
-    <sheet name="Custom Enums" sheetId="14" r:id="rId8"/>
-    <sheet name="Custom Linktypes" sheetId="15" r:id="rId9"/>
-    <sheet name="Custom Protocoltypes" sheetId="16" r:id="rId10"/>
+    <sheet name="Custom Infotypes" sheetId="14" r:id="rId8"/>
+    <sheet name="Custom Types" sheetId="15" r:id="rId9"/>
+    <sheet name="Custom Protocols" sheetId="16" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -49,8 +49,6 @@
   <authors>
     <author>tc={3B0147B9-281D-4130-A8BC-309410749B5B}</author>
     <author>tc={378AC36A-A31E-401E-9A55-70E1232DF5BC}</author>
-    <author>tc={D6BC7333-6530-4BD1-853B-035AED8367A6}</author>
-    <author>tc={8018B6A6-AE10-4F8E-BCB0-2E0A374A5F7F}</author>
   </authors>
   <commentList>
     <comment ref="A3" authorId="0" shapeId="0" xr:uid="{3B0147B9-281D-4130-A8BC-309410749B5B}">
@@ -58,8 +56,7 @@
         <t>[Kommentarthread]
 Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
 Kommentar:
-    The network name.
-Optional string.</t>
+    The network name.</t>
       </text>
     </comment>
     <comment ref="A4" authorId="1" shapeId="0" xr:uid="{378AC36A-A31E-401E-9A55-70E1232DF5BC}">
@@ -67,140 +64,15 @@
         <t>[Kommentarthread]
 Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
 Kommentar:
-    Required connectors.
-Optional comma-separated list of string.</t>
-      </text>
-    </comment>
-    <comment ref="A5" authorId="2" shapeId="0" xr:uid="{D6BC7333-6530-4BD1-853B-035AED8367A6}">
-      <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Optional string</t>
-      </text>
-    </comment>
-    <comment ref="A6" authorId="3" shapeId="0" xr:uid="{8018B6A6-AE10-4F8E-BCB0-2E0A374A5F7F}">
-      <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Optional string</t>
+    Comma-separated list of required connectors</t>
       </text>
     </comment>
   </commentList>
 </comments>
 </file>
 
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>tc={2BE1B318-8F0A-4D91-98E6-F663AC71790C}</author>
-    <author>tc={A6487978-AC63-4DC1-8DBF-E1489D1A1329}</author>
-    <author>tc={DAF89326-DFD8-4953-B5FA-5A1135BB7048}</author>
-    <author>tc={F5AE985E-8139-4FD1-926D-B603986D2AB3}</author>
-    <author>tc={522C9F77-CF7F-4972-8E2F-D7B911B3CA00}</author>
-    <author>tc={39D74A31-E2AE-42FE-8CAD-C0AA71C863D8}</author>
-    <author>tc={638B6463-6700-472E-AE9F-35E6E4638C8C}</author>
-    <author>tc={59D3F605-9DAD-43F9-AC61-0573DE79E336}</author>
-    <author>tc={BE84A17A-DCB9-4278-A4E6-D8061C01FECC}</author>
-    <author>tc={6DEB9449-BF03-4E90-8BE8-E6DC418417CC}</author>
-    <author>tc={4A9EC2E4-39EE-4CAE-A7A0-C51C8A757902}</author>
-  </authors>
-  <commentList>
-    <comment ref="A4" authorId="0" shapeId="0" xr:uid="{2BE1B318-8F0A-4D91-98E6-F663AC71790C}">
-      <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Mandatory int.</t>
-      </text>
-    </comment>
-    <comment ref="B4" authorId="1" shapeId="0" xr:uid="{A6487978-AC63-4DC1-8DBF-E1489D1A1329}">
-      <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Optional string. Default None.</t>
-      </text>
-    </comment>
-    <comment ref="C4" authorId="2" shapeId="0" xr:uid="{DAF89326-DFD8-4953-B5FA-5A1135BB7048}">
-      <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Optional string. Default ROUTER.</t>
-      </text>
-    </comment>
-    <comment ref="D4" authorId="3" shapeId="0" xr:uid="{F5AE985E-8139-4FD1-926D-B603986D2AB3}">
-      <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Optional string, „True“ or „False“. Default „True“.</t>
-      </text>
-    </comment>
-    <comment ref="E4" authorId="4" shapeId="0" xr:uid="{522C9F77-CF7F-4972-8E2F-D7B911B3CA00}">
-      <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Optional string. Default None.</t>
-      </text>
-    </comment>
-    <comment ref="F4" authorId="5" shapeId="0" xr:uid="{39D74A31-E2AE-42FE-8CAD-C0AA71C863D8}">
-      <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Optional comma-separated pair of float. Default None.</t>
-      </text>
-    </comment>
-    <comment ref="G4" authorId="6" shapeId="0" xr:uid="{638B6463-6700-472E-AE9F-35E6E4638C8C}">
-      <text>
-        <t xml:space="preserve">[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Optional comma-separated list of string. Default „all“. </t>
-      </text>
-    </comment>
-    <comment ref="H4" authorId="7" shapeId="0" xr:uid="{59D3F605-9DAD-43F9-AC61-0573DE79E336}">
-      <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Optional float. Default None.</t>
-      </text>
-    </comment>
-    <comment ref="I4" authorId="8" shapeId="0" xr:uid="{BE84A17A-DCB9-4278-A4E6-D8061C01FECC}">
-      <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Optional float. Default None.</t>
-      </text>
-    </comment>
-    <comment ref="J4" authorId="9" shapeId="0" xr:uid="{6DEB9449-BF03-4E90-8BE8-E6DC418417CC}">
-      <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Optional float. Default None.</t>
-      </text>
-    </comment>
-    <comment ref="K4" authorId="10" shapeId="0" xr:uid="{4A9EC2E4-39EE-4CAE-A7A0-C51C8A757902}">
-      <text>
-        <t xml:space="preserve">[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Optional comma-separated pair of string, int. </t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="57">
   <si>
     <t>name</t>
   </si>
@@ -208,6 +80,9 @@
     <t>type</t>
   </si>
   <si>
+    <t>protocols</t>
+  </si>
+  <si>
     <t>length_km</t>
   </si>
   <si>
@@ -292,6 +167,12 @@
     <t>Apps</t>
   </si>
   <si>
+    <t>Custom Types</t>
+  </si>
+  <si>
+    <t>Custom Protocols</t>
+  </si>
+  <si>
     <t>index</t>
   </si>
   <si>
@@ -301,6 +182,12 @@
     <t>Core</t>
   </si>
   <si>
+    <t>pp connector</t>
+  </si>
+  <si>
+    <t>Custom Infotypes</t>
+  </si>
+  <si>
     <t xml:space="preserve">How to use this file </t>
   </si>
   <si>
@@ -322,43 +209,40 @@
     <t xml:space="preserve">It is recommended to do an automated diagnosis run on the ict network auto-generated from this file. </t>
   </si>
   <si>
+    <t>1.1.2preview</t>
+  </si>
+  <si>
     <t>openpyxl_version</t>
   </si>
   <si>
-    <t>pp_pict_connector</t>
-  </si>
-  <si>
-    <t>Custom Enums</t>
-  </si>
-  <si>
-    <t>Custom Linktypes</t>
-  </si>
-  <si>
-    <t>bandwidth_Mbps</t>
-  </si>
-  <si>
-    <t>latency_ms</t>
-  </si>
-  <si>
-    <t>wired</t>
-  </si>
-  <si>
-    <t>protocols</t>
-  </si>
-  <si>
-    <t>ber_per_km</t>
-  </si>
-  <si>
-    <t>Custom Protocoltypes</t>
-  </si>
-  <si>
-    <t>base_package_size_byte</t>
-  </si>
-  <si>
-    <t>payload_size_byte</t>
-  </si>
-  <si>
-    <t>value</t>
+    <t>3.1.5</t>
+  </si>
+  <si>
+    <t>debug</t>
+  </si>
+  <si>
+    <t>pi_pict_connector</t>
+  </si>
+  <si>
+    <t>N1</t>
+  </si>
+  <si>
+    <t>ROUTER</t>
+  </si>
+  <si>
+    <t>True</t>
+  </si>
+  <si>
+    <t>Fiber,Fiber,ADSL8,LTE50</t>
+  </si>
+  <si>
+    <t>N2</t>
+  </si>
+  <si>
+    <t>LAN1000,ADSL8,LTE50</t>
+  </si>
+  <si>
+    <t>4.388, 6.721</t>
   </si>
 </sst>
 </file>
@@ -434,24 +318,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -782,56 +664,10 @@
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="A3" dT="2025-07-21T08:47:53.12" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{3B0147B9-281D-4130-A8BC-309410749B5B}">
-    <text>The network name.
-Optional string.</text>
+    <text>The network name.</text>
   </threadedComment>
   <threadedComment ref="A4" dT="2025-07-21T08:48:29.39" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{378AC36A-A31E-401E-9A55-70E1232DF5BC}">
-    <text>Required connectors.
-Optional comma-separated list of string.</text>
-  </threadedComment>
-  <threadedComment ref="A5" dT="2025-08-01T09:45:52.28" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{D6BC7333-6530-4BD1-853B-035AED8367A6}">
-    <text>Optional string</text>
-  </threadedComment>
-  <threadedComment ref="A6" dT="2025-08-01T09:46:07.43" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{8018B6A6-AE10-4F8E-BCB0-2E0A374A5F7F}">
-    <text>Optional string</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
-<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A4" dT="2025-08-01T09:46:42.38" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{2BE1B318-8F0A-4D91-98E6-F663AC71790C}">
-    <text>Mandatory int.</text>
-  </threadedComment>
-  <threadedComment ref="B4" dT="2025-08-01T09:46:54.51" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{A6487978-AC63-4DC1-8DBF-E1489D1A1329}">
-    <text>Optional string. Default None.</text>
-  </threadedComment>
-  <threadedComment ref="C4" dT="2025-08-01T09:47:18.39" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{DAF89326-DFD8-4953-B5FA-5A1135BB7048}">
-    <text>Optional string. Default ROUTER.</text>
-  </threadedComment>
-  <threadedComment ref="D4" dT="2025-08-01T09:47:56.77" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{F5AE985E-8139-4FD1-926D-B603986D2AB3}">
-    <text>Optional string, „True“ or „False“. Default „True“.</text>
-  </threadedComment>
-  <threadedComment ref="E4" dT="2025-08-01T09:48:55.54" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{522C9F77-CF7F-4972-8E2F-D7B911B3CA00}">
-    <text>Optional string. Default None.</text>
-  </threadedComment>
-  <threadedComment ref="F4" dT="2025-08-01T09:49:32.36" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{39D74A31-E2AE-42FE-8CAD-C0AA71C863D8}">
-    <text>Optional comma-separated pair of float. Default None.</text>
-  </threadedComment>
-  <threadedComment ref="G4" dT="2025-08-01T09:49:52.86" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{638B6463-6700-472E-AE9F-35E6E4638C8C}">
-    <text xml:space="preserve">Optional comma-separated list of string. Default „all“. </text>
-  </threadedComment>
-  <threadedComment ref="H4" dT="2025-08-01T09:50:07.55" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{59D3F605-9DAD-43F9-AC61-0573DE79E336}">
-    <text>Optional float. Default None.</text>
-  </threadedComment>
-  <threadedComment ref="I4" dT="2025-08-01T09:50:12.64" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{BE84A17A-DCB9-4278-A4E6-D8061C01FECC}">
-    <text>Optional float. Default None.</text>
-  </threadedComment>
-  <threadedComment ref="J4" dT="2025-08-01T09:50:17.21" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{6DEB9449-BF03-4E90-8BE8-E6DC418417CC}">
-    <text>Optional float. Default None.</text>
-  </threadedComment>
-  <threadedComment ref="K4" dT="2025-08-01T09:50:57.93" personId="{5E3593F0-A5F3-449A-9956-7F9F1B4BBD0B}" id="{4A9EC2E4-39EE-4CAE-A7A0-C51C8A757902}">
-    <text xml:space="preserve">Optional comma-separated pair of string, int. </text>
+    <text>Comma-separated list of required connectors</text>
   </threadedComment>
 </ThreadedComments>
 </file>
@@ -843,39 +679,39 @@
   <sheetData>
     <row r="1" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -885,57 +721,15 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84425F92-1B1F-4810-8ABA-3011E45EA319}">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="3" max="3" width="23.7109375" customWidth="1"/>
-    <col min="4" max="4" width="76.140625" customWidth="1"/>
-    <col min="5" max="5" width="45.28515625" customWidth="1"/>
-    <col min="6" max="6" width="47.7109375" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:1" s="1" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B3" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B3:F3"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -953,7 +747,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -962,23 +756,33 @@
       <c r="A3" t="s">
         <v>0</v>
       </c>
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="7"/>
+        <v>23</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="6"/>
+        <v>46</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>47</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -987,7 +791,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F502733A-EE70-40FB-9F5D-B6735209FF83}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F502733A-EE70-40FB-9F5D-B6735209FF83}">
   <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -997,13 +801,13 @@
     <col min="4" max="6" width="11.42578125" customWidth="1"/>
     <col min="7" max="7" width="23.140625" customWidth="1"/>
     <col min="8" max="10" width="11.42578125" customWidth="1"/>
-    <col min="11" max="11" width="19.85546875" customWidth="1"/>
+    <col min="11" max="11" width="15.42578125" customWidth="1"/>
     <col min="12" max="16384" width="11.42578125" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1017,24 +821,25 @@
       <c r="K1" s="1"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
+      <c r="A3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
       <c r="K3" s="2" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>0</v>
@@ -1043,42 +848,90 @@
         <v>1</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>4</v>
-      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H5" s="8"/>
+      <c r="A5">
+        <v>0</v>
+      </c>
+      <c r="B5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H5" s="10">
+        <v>1E-3</v>
+      </c>
+      <c r="I5">
+        <v>2000</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H6" s="8"/>
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H6" s="10">
+        <v>2E-3</v>
+      </c>
+      <c r="I6">
+        <v>1000</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="A3:J3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1087,77 +940,11 @@
   <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="7" width="11.42578125" customWidth="1"/>
-    <col min="8" max="12" width="0" hidden="1" customWidth="1"/>
+    <col min="1" max="12" width="11.42578125" customWidth="1"/>
     <col min="13" max="16384" width="11.42578125" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B3:G3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAF5917D-01F4-4445-A259-36CFC198F1F3}">
-  <dimension ref="A1:XFB4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="8" width="11.42578125" customWidth="1"/>
-    <col min="9" max="9" width="18.5703125" customWidth="1"/>
-    <col min="10" max="11" width="0" hidden="1" customWidth="1"/>
-    <col min="12" max="16382" width="11.42578125" hidden="1"/>
-    <col min="16383" max="16383" width="2.5703125" hidden="1" customWidth="1"/>
-    <col min="16384" max="16384" width="2.5703125" hidden="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>27</v>
       </c>
@@ -1169,24 +956,31 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>0</v>
@@ -1195,29 +989,120 @@
         <v>1</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="G4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="I3:L3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAF5917D-01F4-4445-A259-36CFC198F1F3}">
+  <dimension ref="A1:L4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="9" width="11.42578125" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" customWidth="1"/>
+    <col min="11" max="12" width="0" hidden="1" customWidth="1"/>
+    <col min="13" max="16384" width="11.42578125" hidden="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="A1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>17</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>18</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>2</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="J4" s="5"/>
+        <v>3</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>5</v>
+      </c>
       <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1236,7 +1121,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1250,58 +1135,59 @@
       <c r="K1" s="1"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B3" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
+      <c r="A3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4" s="4" t="s">
         <v>21</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>20</v>
       </c>
       <c r="L4" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="A3:K3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1309,16 +1195,16 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9747E980-AD4A-433D-B25D-167EB1EBAE1A}">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="16384" width="11.42578125" hidden="1"/>
+    <col min="1" max="7" width="11.42578125" customWidth="1"/>
+    <col min="8" max="16384" width="11.42578125" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1326,30 +1212,21 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>0</v>
@@ -1358,34 +1235,21 @@
         <v>1</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="H3:K3"/>
-    <mergeCell ref="B3:G3"/>
+  <mergeCells count="1">
+    <mergeCell ref="A3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1393,135 +1257,35 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A44E78A-AEC8-469F-B4D1-78F61DE32AAE}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:1" s="1" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="12"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="E4" s="11"/>
+        <v>37</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B3:D3"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB02342F-BC9A-4A38-B4AC-80F6821C570F}">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="3" max="3" width="19.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17.140625" customWidth="1"/>
-    <col min="6" max="6" width="33" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:1" s="1" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B3" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B3:J3"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="f96729ad-c324-4e99-8ea2-5eb7509c173e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e711f135-e4e6-4e79-b81d-a0615d74429e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100EEC6A9F56DB8DE4E994ECFB7CFB7F060" ma:contentTypeVersion="10" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="9620f1347f6a5fb9ad440f9c98bddfff">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e711f135-e4e6-4e79-b81d-a0615d74429e" xmlns:ns3="f96729ad-c324-4e99-8ea2-5eb7509c173e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0567a5e3a89b686b1bdd445dd792ccfb" ns2:_="" ns3:_="">
     <xsd:import namespace="e711f135-e4e6-4e79-b81d-a0615d74429e"/>
@@ -1710,32 +1474,27 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="f96729ad-c324-4e99-8ea2-5eb7509c173e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e711f135-e4e6-4e79-b81d-a0615d74429e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B6CB480-C731-4173-8ADD-4C715894D07C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA58780A-0059-4AB4-9F66-F670DB764EE0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="f96729ad-c324-4e99-8ea2-5eb7509c173e"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="e711f135-e4e6-4e79-b81d-a0615d74429e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{586680BC-277B-44FC-B0E0-A4251335AB07}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1752,4 +1511,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B6CB480-C731-4173-8ADD-4C715894D07C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA58780A-0059-4AB4-9F66-F670DB764EE0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="f96729ad-c324-4e99-8ea2-5eb7509c173e"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="e711f135-e4e6-4e79-b81d-a0615d74429e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>